<commit_message>
Changes in Matplotlib, Numpy, Pandas and new files in Sklearn
</commit_message>
<xml_diff>
--- a/Pandas/students_data2.xlsx
+++ b/Pandas/students_data2.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:D4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,6 +436,11 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>City</t>
         </is>
       </c>
@@ -449,6 +454,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Alice</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>New York</t>
         </is>
       </c>
@@ -462,6 +472,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Bob</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>Los Angeles</t>
         </is>
       </c>
@@ -474,6 +489,11 @@
         <v>22</v>
       </c>
       <c r="C4" t="inlineStr">
+        <is>
+          <t>Charlie</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
         <is>
           <t>Chicago</t>
         </is>

</xml_diff>